<commit_message>
Revised Open-Loop Boost test results with new methodology
</commit_message>
<xml_diff>
--- a/OL test results.xlsx
+++ b/OL test results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderward/Downloads/UNI/3rd Year/311/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexanderward/Downloads/UNI/3rd Year/311/PR2/Scope Outputs/OL TEST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D575E828-34C7-5D46-AE07-36DC6DAA311A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3B96677-78E3-6D48-96C2-DD2BD4B5F183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2780" yWindow="1500" windowWidth="28040" windowHeight="17440" xr2:uid="{F7317023-7B2B-674E-B17E-7765013A1353}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>Vin</t>
   </si>
@@ -60,6 +60,24 @@
   </si>
   <si>
     <t>Required DC (Inverted-Real)</t>
+  </si>
+  <si>
+    <t>Vin (PCB)</t>
+  </si>
+  <si>
+    <t>Iin (PS)</t>
+  </si>
+  <si>
+    <t>Vout (PCB)</t>
+  </si>
+  <si>
+    <t>Iout (EL)</t>
+  </si>
+  <si>
+    <t>Initial Results</t>
+  </si>
+  <si>
+    <t>Input and Output GNDS connected and manually calculated PCB power so as to not include external cable loss in PCB performance</t>
   </si>
 </sst>
 </file>
@@ -103,9 +121,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -441,357 +460,774 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{309630EC-AF18-034A-91E8-0DCF7CCEF4D1}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" customWidth="1"/>
-    <col min="5" max="5" width="23.33203125" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D3" t="s">
         <v>6</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E3" t="s">
         <v>7</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F3" t="s">
         <v>2</v>
       </c>
-      <c r="G1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2">
-        <v>2.5</v>
-      </c>
-      <c r="B2">
-        <v>4.7</v>
-      </c>
-      <c r="C2">
-        <v>5</v>
-      </c>
-      <c r="D2">
-        <v>25</v>
-      </c>
-      <c r="E2">
-        <f>100-D2</f>
-        <v>75</v>
-      </c>
-      <c r="F2">
-        <v>6.95</v>
-      </c>
-      <c r="G2">
-        <v>3.3</v>
-      </c>
-      <c r="H2" s="1">
-        <f>G2/F2</f>
-        <v>0.47482014388489208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3">
-        <v>2.5</v>
-      </c>
-      <c r="B3">
-        <v>5</v>
-      </c>
-      <c r="C3">
-        <v>16.25</v>
-      </c>
-      <c r="D3">
-        <v>41</v>
-      </c>
-      <c r="E3">
-        <f t="shared" ref="E3:E12" si="0">100-D3</f>
-        <v>59</v>
-      </c>
-      <c r="F3">
-        <v>1.71</v>
-      </c>
-      <c r="G3">
-        <v>1.35</v>
-      </c>
-      <c r="H3" s="1">
-        <f t="shared" ref="H3:H12" si="1">G3/F3</f>
-        <v>0.78947368421052644</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>2.5</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>4.7</v>
       </c>
       <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>25</v>
+      </c>
+      <c r="E4">
+        <f>100-D4</f>
+        <v>75</v>
+      </c>
+      <c r="F4">
+        <v>6.95</v>
+      </c>
+      <c r="I4" t="s">
+        <v>3</v>
+      </c>
+      <c r="J4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2.5</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>16.25</v>
+      </c>
+      <c r="D5">
+        <v>41</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E14" si="0">100-D5</f>
+        <v>59</v>
+      </c>
+      <c r="F5">
+        <v>1.71</v>
+      </c>
+      <c r="I5">
+        <v>3.3</v>
+      </c>
+      <c r="J5" s="1">
+        <f>I5/F4</f>
+        <v>0.47482014388489208</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2.5</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
         <v>27.5</v>
       </c>
-      <c r="D4">
+      <c r="D6">
         <v>43</v>
       </c>
-      <c r="E4">
+      <c r="E6">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
-      <c r="F4">
+      <c r="F6">
         <v>1</v>
       </c>
-      <c r="G4">
-        <v>0.83</v>
-      </c>
-      <c r="H4" s="1">
-        <f t="shared" si="1"/>
-        <v>0.83</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5">
+      <c r="I6">
+        <v>1.35</v>
+      </c>
+      <c r="J6" s="1">
+        <f>I6/F5</f>
+        <v>0.78947368421052644</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>2.5</v>
       </c>
-      <c r="B5">
-        <v>5</v>
-      </c>
-      <c r="C5">
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
         <v>38.75</v>
       </c>
-      <c r="D5">
+      <c r="D7">
         <v>44</v>
       </c>
-      <c r="E5">
+      <c r="E7">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="F5">
+      <c r="F7">
         <v>0.7</v>
       </c>
-      <c r="G5">
-        <v>0.6</v>
-      </c>
-      <c r="H5" s="1">
-        <f t="shared" si="1"/>
-        <v>0.85714285714285721</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6">
+      <c r="I7">
+        <v>0.83</v>
+      </c>
+      <c r="J7" s="1">
+        <f>I7/F6</f>
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>2.5</v>
       </c>
-      <c r="B6">
-        <v>5</v>
-      </c>
-      <c r="C6">
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8">
         <v>50</v>
       </c>
-      <c r="D6">
+      <c r="D8">
         <v>44</v>
       </c>
-      <c r="E6">
+      <c r="E8">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
-      <c r="F6">
+      <c r="F8">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G6">
+      <c r="I8">
+        <v>0.6</v>
+      </c>
+      <c r="J8" s="1">
+        <f>I8/F7</f>
+        <v>0.85714285714285721</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I9">
         <v>0.48</v>
       </c>
-      <c r="H6" s="1">
-        <f t="shared" si="1"/>
+      <c r="J9" s="1">
+        <f>I9/F8</f>
         <v>0.87272727272727257</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>3.5</v>
       </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8">
-        <v>5</v>
-      </c>
-      <c r="D8">
+      <c r="B10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
         <v>55</v>
       </c>
-      <c r="E8">
+      <c r="E10">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="F8">
+      <c r="F10">
         <v>5.16</v>
       </c>
-      <c r="G8">
-        <v>3.4</v>
-      </c>
-      <c r="H8" s="1">
-        <f>G8/F8</f>
-        <v>0.65891472868217049</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9">
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>3.5</v>
       </c>
-      <c r="B9">
-        <v>5</v>
-      </c>
-      <c r="C9">
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11">
         <v>16.25</v>
       </c>
-      <c r="D9">
+      <c r="D11">
         <v>61</v>
       </c>
-      <c r="E9">
+      <c r="E11">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="F9">
+      <c r="F11">
         <v>1.61</v>
       </c>
-      <c r="G9">
-        <v>1.32</v>
-      </c>
-      <c r="H9" s="1">
-        <f>G9/F9</f>
-        <v>0.81987577639751552</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10">
+      <c r="I11">
+        <v>3.4</v>
+      </c>
+      <c r="J11" s="1">
+        <f>I11/F10</f>
+        <v>0.65891472868217049</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12">
         <v>3.5</v>
       </c>
-      <c r="B10">
-        <v>5</v>
-      </c>
-      <c r="C10">
+      <c r="B12">
+        <v>5</v>
+      </c>
+      <c r="C12">
         <v>27.5</v>
       </c>
-      <c r="D10">
+      <c r="D12">
         <v>63</v>
       </c>
-      <c r="E10">
+      <c r="E12">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="F10">
+      <c r="F12">
         <v>0.97</v>
       </c>
-      <c r="G10">
-        <v>0.84</v>
-      </c>
-      <c r="H10" s="1">
-        <f t="shared" si="1"/>
-        <v>0.865979381443299</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11">
+      <c r="I12">
+        <v>1.32</v>
+      </c>
+      <c r="J12" s="1">
+        <f>I12/F11</f>
+        <v>0.81987577639751552</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13">
         <v>3.5</v>
       </c>
-      <c r="B11">
-        <v>5</v>
-      </c>
-      <c r="C11">
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13">
         <v>38.75</v>
       </c>
-      <c r="D11">
+      <c r="D13">
         <v>64</v>
       </c>
-      <c r="E11">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="F11">
+      <c r="F13">
         <v>0.71</v>
       </c>
-      <c r="G11">
-        <v>0.62</v>
-      </c>
-      <c r="H11" s="1">
-        <f t="shared" si="1"/>
-        <v>0.87323943661971837</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12">
+      <c r="I13">
+        <v>0.84</v>
+      </c>
+      <c r="J13" s="1">
+        <f>I13/F12</f>
+        <v>0.865979381443299</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14">
         <v>3.5</v>
       </c>
-      <c r="B12">
-        <v>5</v>
-      </c>
-      <c r="C12">
+      <c r="B14">
+        <v>5</v>
+      </c>
+      <c r="C14">
         <v>50</v>
       </c>
-      <c r="D12">
+      <c r="D14">
         <v>65</v>
       </c>
-      <c r="E12">
+      <c r="E14">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="F12">
+      <c r="F14">
         <v>0.55000000000000004</v>
       </c>
-      <c r="G12">
+      <c r="I14">
+        <v>0.62</v>
+      </c>
+      <c r="J14" s="1">
+        <f>I14/F13</f>
+        <v>0.87323943661971837</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I16">
         <v>0.49</v>
       </c>
-      <c r="H12" s="1">
+      <c r="J16" s="1">
+        <f>I16/F14</f>
+        <v>0.89090909090909087</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>7</v>
+      </c>
+      <c r="D20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
+        <v>2</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" t="s">
+        <v>3</v>
+      </c>
+      <c r="J20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>5</v>
+      </c>
+      <c r="B21">
+        <v>37</v>
+      </c>
+      <c r="C21">
+        <f>100-B21</f>
+        <v>63</v>
+      </c>
+      <c r="D21">
+        <v>2.52</v>
+      </c>
+      <c r="E21">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="F21">
+        <f>E21*D21</f>
+        <v>6.1236000000000006</v>
+      </c>
+      <c r="G21">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="H21">
+        <v>0.93</v>
+      </c>
+      <c r="I21">
+        <f>G21*H21</f>
+        <v>4.6314000000000011</v>
+      </c>
+      <c r="J21" s="1">
+        <f>I21/F21</f>
+        <v>0.75631981187536756</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>16.25</v>
+      </c>
+      <c r="B22">
+        <v>41</v>
+      </c>
+      <c r="C22">
+        <f t="shared" ref="C22:C25" si="1">100-B22</f>
+        <v>59</v>
+      </c>
+      <c r="D22">
+        <v>2.5</v>
+      </c>
+      <c r="E22">
+        <v>0.72</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22:F31" si="2">E22*D22</f>
+        <v>1.7999999999999998</v>
+      </c>
+      <c r="G22">
+        <v>5.0599999999999996</v>
+      </c>
+      <c r="H22">
+        <v>0.30499999999999999</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22:I31" si="3">G22*H22</f>
+        <v>1.5432999999999999</v>
+      </c>
+      <c r="J22" s="1">
+        <f t="shared" ref="J22:J31" si="4">I22/F22</f>
+        <v>0.85738888888888887</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>27.5</v>
+      </c>
+      <c r="B23">
+        <v>44</v>
+      </c>
+      <c r="C23">
         <f t="shared" si="1"/>
-        <v>0.89090909090909087</v>
-      </c>
-    </row>
-    <row r="30" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H31" s="1"/>
-    </row>
-    <row r="32" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H32" s="1"/>
-    </row>
-    <row r="33" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H33" s="1"/>
-    </row>
-    <row r="34" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H34" s="1"/>
-    </row>
-    <row r="35" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H35" s="1"/>
-    </row>
-    <row r="36" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H36" s="1"/>
-    </row>
-    <row r="37" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H37" s="1"/>
-    </row>
-    <row r="38" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H38" s="1"/>
-    </row>
-    <row r="39" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H39" s="1"/>
-    </row>
-    <row r="40" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H40" s="1"/>
-    </row>
-    <row r="41" spans="8:8" x14ac:dyDescent="0.2">
-      <c r="H41" s="1"/>
+        <v>56</v>
+      </c>
+      <c r="D23">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="E23">
+        <v>0.40400000000000003</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="2"/>
+        <v>1.0140400000000001</v>
+      </c>
+      <c r="G23">
+        <v>5.01</v>
+      </c>
+      <c r="H23">
+        <v>0.18</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="3"/>
+        <v>0.90179999999999993</v>
+      </c>
+      <c r="J23" s="1">
+        <f t="shared" si="4"/>
+        <v>0.88931403100469397</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24">
+        <v>38.75</v>
+      </c>
+      <c r="B24">
+        <v>45</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="1"/>
+        <v>55</v>
+      </c>
+      <c r="D24">
+        <v>2.4900000000000002</v>
+      </c>
+      <c r="E24">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="2"/>
+        <v>0.69720000000000015</v>
+      </c>
+      <c r="G24">
+        <v>4.96</v>
+      </c>
+      <c r="H24">
+        <v>0.125</v>
+      </c>
+      <c r="I24">
+        <f t="shared" si="3"/>
+        <v>0.62</v>
+      </c>
+      <c r="J24" s="1">
+        <f t="shared" si="4"/>
+        <v>0.88927137119908184</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>50</v>
+      </c>
+      <c r="B25">
+        <v>45</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="1"/>
+        <v>55</v>
+      </c>
+      <c r="D25">
+        <v>2.5</v>
+      </c>
+      <c r="E25">
+        <v>0.22</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="2"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G25">
+        <v>4.99</v>
+      </c>
+      <c r="H25">
+        <v>0.1</v>
+      </c>
+      <c r="I25">
+        <f t="shared" si="3"/>
+        <v>0.49900000000000005</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" si="4"/>
+        <v>0.90727272727272734</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>5</v>
+      </c>
+      <c r="B27">
+        <v>58</v>
+      </c>
+      <c r="C27">
+        <f t="shared" ref="C27:C31" si="5">100-B27</f>
+        <v>42</v>
+      </c>
+      <c r="D27">
+        <v>3.51</v>
+      </c>
+      <c r="E27">
+        <v>1.65</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="2"/>
+        <v>5.7914999999999992</v>
+      </c>
+      <c r="G27">
+        <v>5</v>
+      </c>
+      <c r="H27">
+        <v>0.98</v>
+      </c>
+      <c r="I27">
+        <f t="shared" si="3"/>
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" si="4"/>
+        <v>0.84606751273417957</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>16.25</v>
+      </c>
+      <c r="B28">
+        <v>63</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="5"/>
+        <v>37</v>
+      </c>
+      <c r="D28">
+        <v>3.4990000000000001</v>
+      </c>
+      <c r="E28">
+        <v>0.49199999999999999</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="2"/>
+        <v>1.721508</v>
+      </c>
+      <c r="G28">
+        <v>4.9800000000000004</v>
+      </c>
+      <c r="H28">
+        <v>0.3</v>
+      </c>
+      <c r="I28">
+        <f t="shared" si="3"/>
+        <v>1.494</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="4"/>
+        <v>0.86784377417938219</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>27.5</v>
+      </c>
+      <c r="B29">
+        <v>63</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="5"/>
+        <v>37</v>
+      </c>
+      <c r="D29">
+        <v>3.4969999999999999</v>
+      </c>
+      <c r="E29">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="2"/>
+        <v>1.01413</v>
+      </c>
+      <c r="G29">
+        <v>5.05</v>
+      </c>
+      <c r="H29">
+        <v>0.18</v>
+      </c>
+      <c r="I29">
+        <f t="shared" si="3"/>
+        <v>0.90899999999999992</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" si="4"/>
+        <v>0.89633478942541878</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>38.75</v>
+      </c>
+      <c r="B30">
+        <v>64</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="5"/>
+        <v>36</v>
+      </c>
+      <c r="D30">
+        <v>3.51</v>
+      </c>
+      <c r="E30">
+        <v>0.2</v>
+      </c>
+      <c r="F30">
+        <f t="shared" si="2"/>
+        <v>0.70199999999999996</v>
+      </c>
+      <c r="G30">
+        <v>5.01</v>
+      </c>
+      <c r="H30">
+        <v>0.127</v>
+      </c>
+      <c r="I30">
+        <f t="shared" si="3"/>
+        <v>0.63627</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="4"/>
+        <v>0.90636752136752141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>50</v>
+      </c>
+      <c r="B31">
+        <v>65</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="5"/>
+        <v>35</v>
+      </c>
+      <c r="D31">
+        <v>3.51</v>
+      </c>
+      <c r="E31">
+        <v>0.152</v>
+      </c>
+      <c r="F31">
+        <f t="shared" si="2"/>
+        <v>0.53351999999999999</v>
+      </c>
+      <c r="G31">
+        <v>4.96</v>
+      </c>
+      <c r="H31">
+        <v>0.1</v>
+      </c>
+      <c r="I31">
+        <f t="shared" si="3"/>
+        <v>0.496</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="4"/>
+        <v>0.92967461388514017</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L32" s="1"/>
+    </row>
+    <row r="33" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L33" s="1"/>
+    </row>
+    <row r="34" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L34" s="1"/>
+    </row>
+    <row r="35" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L35" s="1"/>
+    </row>
+    <row r="36" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L36" s="1"/>
+    </row>
+    <row r="37" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L37" s="1"/>
+    </row>
+    <row r="38" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L38" s="1"/>
+    </row>
+    <row r="39" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L39" s="1"/>
+    </row>
+    <row r="40" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L40" s="1"/>
+    </row>
+    <row r="41" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L41" s="1"/>
+    </row>
+    <row r="42" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L42" s="1"/>
+    </row>
+    <row r="43" spans="12:12" x14ac:dyDescent="0.2">
+      <c r="L43" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>